<commit_message>
BR-002: point the guide at the Speak Up help center link
Renaming the help center in the sandbox moved its address from
/helpcenter/WhistleblowingReporting to /helpcenter/SpeakUp, and the old
link now shows an error page. The guide uses the new link, and BR-002
records the change so production links get replaced too.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/WB-Requirements-and-SLA-Template-v1.4.xlsx
+++ b/docs/WB-Requirements-and-SLA-Template-v1.4.xlsx
@@ -734,7 +734,7 @@
     <t>New</t>
   </si>
   <si>
-    <t>Portal name and emails are configuration only. The portal link does not change, so links already shared keep working.</t>
+    <t>Sandbox, 21/10/2026: done - project, portal and help center renamed, emails and user guide (v1.2) updated. The help center address changed with it, from /helpcenter/WhistleblowingReporting to /helpcenter/SpeakUp: the old link no longer opens the form, so every published link (intranet, emails, posters, QR codes) must be replaced when this goes to production. Production: not started.</t>
   </si>
   <si>
     <t>Anonymity notice next to the anonymous option</t>
@@ -5755,7 +5755,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="str">
         <f t="shared" ref="A7:A38" si="0">IF(C7="","","BR-"&amp;TEXT(ROW()-5,"000"))</f>
         <v>BR-002</v>

</xml_diff>

<commit_message>
Requirements template: 'Done in sandbox' status; BR-002 set to it
'Implemented' stays for live in production, so the tracker does not
claim more than has been built.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/WB-Requirements-and-SLA-Template-v1.4.xlsx
+++ b/docs/WB-Requirements-and-SLA-Template-v1.4.xlsx
@@ -27,7 +27,7 @@
     <definedName name="JiraField">Lists!$N$2:$N$16</definedName>
     <definedName name="Priority">Lists!$B$2:$B$5</definedName>
     <definedName name="ReportCategory">Lists!$D$2:$D$12</definedName>
-    <definedName name="ReqStatus">Lists!$C$2:$C$6</definedName>
+    <definedName name="ReqStatus">Lists!$C$2:$C$7</definedName>
     <definedName name="Requesters">Lists!$K$2:$K$6</definedName>
     <definedName name="ServiceNames">'Service Catalog'!$C$6:$C$66</definedName>
     <definedName name="Severity">Lists!$E$2:$E$6</definedName>
@@ -271,7 +271,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>Filled in jointly with Ejada during review.</t>
+          <t>Filled in jointly with Ejada during review. Done in sandbox = built and checked in the sandbox, not yet in production. Implemented = live in production.</t>
         </r>
       </text>
     </comment>
@@ -346,7 +346,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="398">
   <si>
     <t>Whistleblowing Reporting Portal - Requirements Template</t>
   </si>
@@ -731,19 +731,22 @@
     <t>The portal, the emails and the user guide show "Speak Up"; "Whistleblowing Reporting Portal" no longer appears anywhere a reporter or staff member can see it.</t>
   </si>
   <si>
+    <t>Done in sandbox</t>
+  </si>
+  <si>
+    <t>Sandbox, 21/10/2026: done - project, portal and help center renamed, emails and user guide (v1.2) updated. The help center address changed with it, from /helpcenter/WhistleblowingReporting to /helpcenter/SpeakUp: the old link no longer opens the form, so every published link (intranet, emails, posters, QR codes) must be replaced when this goes to production. Production: not started.</t>
+  </si>
+  <si>
+    <t>Anonymity notice next to the anonymous option</t>
+  </si>
+  <si>
+    <t>Next to the anonymity selection option on the reporting form, show this statement: "Please note that choosing to remain anonymous may limit our ability to clarify facts or follow up with you during the investigation."</t>
+  </si>
+  <si>
+    <t>Opening the reporting form shows the statement, word for word, directly next to the anonymity option, before the reporter submits.</t>
+  </si>
+  <si>
     <t>New</t>
-  </si>
-  <si>
-    <t>Sandbox, 21/10/2026: done - project, portal and help center renamed, emails and user guide (v1.2) updated. The help center address changed with it, from /helpcenter/WhistleblowingReporting to /helpcenter/SpeakUp: the old link no longer opens the form, so every published link (intranet, emails, posters, QR codes) must be replaced when this goes to production. Production: not started.</t>
-  </si>
-  <si>
-    <t>Anonymity notice next to the anonymous option</t>
-  </si>
-  <si>
-    <t>Next to the anonymity selection option on the reporting form, show this statement: "Please note that choosing to remain anonymous may limit our ability to clarify facts or follow up with you during the investigation."</t>
-  </si>
-  <si>
-    <t>Opening the reporting form shows the statement, word for word, directly next to the anonymity option, before the reporter submits.</t>
   </si>
   <si>
     <t>Shown as the help text of the anonymity option. Arabic text to confirm: "يرجى العلم بأن اختيار عدم الإفصاح عن هويتك قد يحدّ من قدرتنا على استيضاح الوقائع أو المتابعة معك أثناء التحقيق."</t>
@@ -5807,10 +5810,10 @@
       </c>
       <c r="J8" s="17"/>
       <c r="K8" s="14" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="L8" s="14" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="92.4" x14ac:dyDescent="0.3">
@@ -5822,24 +5825,24 @@
         <v>119</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>
       <c r="I9" s="14" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J9" s="17"/>
       <c r="K9" s="14" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="409.6" x14ac:dyDescent="0.3">
@@ -5851,24 +5854,24 @@
         <v>119</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E10" s="14"/>
       <c r="F10" s="14"/>
       <c r="G10" s="14"/>
       <c r="H10" s="14"/>
       <c r="I10" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J10" s="17"/>
       <c r="K10" s="14" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="L10" s="14" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="184.8" x14ac:dyDescent="0.3">
@@ -5877,27 +5880,27 @@
         <v>BR-006</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
       <c r="I11" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J11" s="17"/>
       <c r="K11" s="14" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="158.4" x14ac:dyDescent="0.3">
@@ -5906,27 +5909,27 @@
         <v>BR-007</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E12" s="14"/>
       <c r="F12" s="14"/>
       <c r="G12" s="14"/>
       <c r="H12" s="14"/>
       <c r="I12" s="14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J12" s="17"/>
       <c r="K12" s="14" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="L12" s="14" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -6890,7 +6893,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="30" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
@@ -6899,7 +6902,7 @@
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -6908,27 +6911,27 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>97</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
@@ -6936,16 +6939,16 @@
         <v>1</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F6" s="14"/>
     </row>
@@ -6954,16 +6957,16 @@
         <v>2</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F7" s="14"/>
     </row>
@@ -6972,13 +6975,13 @@
         <v>3</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E8" s="19" t="s">
         <v>68</v>
@@ -6990,16 +6993,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F9" s="14"/>
     </row>
@@ -7011,10 +7014,10 @@
         <v>108</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E10" s="19" t="s">
         <v>68</v>
@@ -7026,16 +7029,16 @@
         <v>6</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F11" s="14"/>
     </row>
@@ -7044,16 +7047,16 @@
         <v>7</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F12" s="14"/>
     </row>
@@ -7062,16 +7065,16 @@
         <v>8</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F13" s="14"/>
     </row>
@@ -7080,19 +7083,19 @@
         <v>9</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C14" s="19" t="s">
         <v>68</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
@@ -7100,13 +7103,13 @@
         <v>10</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E15" s="21" t="s">
         <v>68</v>
@@ -7118,13 +7121,13 @@
         <v>11</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C16" s="19" t="s">
         <v>68</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E16" s="19" t="s">
         <v>68</v>
@@ -7159,7 +7162,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="30" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
@@ -7168,7 +7171,7 @@
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -7177,27 +7180,27 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>97</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
@@ -7205,16 +7208,16 @@
         <v>1</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F6" s="14"/>
     </row>
@@ -7223,16 +7226,16 @@
         <v>2</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F7" s="14"/>
     </row>
@@ -7241,16 +7244,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>68</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F8" s="14"/>
     </row>
@@ -7259,16 +7262,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F9" s="14"/>
     </row>
@@ -7277,13 +7280,13 @@
         <v>5</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E10" s="19" t="s">
         <v>68</v>
@@ -7295,16 +7298,16 @@
         <v>6</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F11" s="14"/>
     </row>
@@ -7313,16 +7316,16 @@
         <v>7</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>68</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F12" s="14"/>
     </row>
@@ -7331,16 +7334,16 @@
         <v>8</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F13" s="14"/>
     </row>
@@ -7352,10 +7355,10 @@
         <v>108</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E14" s="19" t="s">
         <v>68</v>
@@ -7367,13 +7370,13 @@
         <v>10</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E15" s="21" t="s">
         <v>68</v>
@@ -7385,13 +7388,13 @@
         <v>11</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E16" s="19" t="s">
         <v>68</v>
@@ -7444,7 +7447,7 @@
   <sheetData>
     <row r="1" spans="1:27" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="30" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
@@ -7474,7 +7477,7 @@
     </row>
     <row r="2" spans="1:27" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -7504,144 +7507,144 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="S5" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="T5" s="10" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="U5" s="10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="V5" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="W5" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="X5" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="Y5" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="Z5" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AA5" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I6" s="11">
         <v>2</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L6" s="25">
         <v>0.75</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="N6" s="11"/>
       <c r="O6" s="11">
         <v>0</v>
       </c>
       <c r="P6" s="11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q6" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="R6" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="S6" s="11">
         <v>1</v>
@@ -7654,7 +7657,7 @@
       <c r="Y6" s="11"/>
       <c r="Z6" s="11"/>
       <c r="AA6" s="11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="26.4" x14ac:dyDescent="0.3">
@@ -7663,34 +7666,34 @@
         <v>SLA-02</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G7" s="26" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H7" s="26" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I7" s="26">
         <v>2</v>
       </c>
       <c r="J7" s="26" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K7" s="26" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L7" s="27"/>
       <c r="M7" s="26"/>
@@ -7699,13 +7702,13 @@
         <v>0</v>
       </c>
       <c r="P7" s="26" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q7" s="26" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="R7" s="26" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="S7" s="26"/>
       <c r="T7" s="26"/>
@@ -7716,7 +7719,7 @@
       <c r="Y7" s="26"/>
       <c r="Z7" s="26"/>
       <c r="AA7" s="26" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
@@ -9694,7 +9697,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="30" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
@@ -9705,7 +9708,7 @@
     </row>
     <row r="2" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -9716,67 +9719,67 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F6" s="11" t="s">
         <v>89</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
@@ -9787,10 +9790,10 @@
     </row>
     <row r="8" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="14"/>
@@ -9801,10 +9804,10 @@
     </row>
     <row r="9" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
@@ -9815,10 +9818,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
@@ -9829,10 +9832,10 @@
     </row>
     <row r="11" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
@@ -9843,10 +9846,10 @@
     </row>
     <row r="12" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
@@ -9857,10 +9860,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
@@ -9871,10 +9874,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
@@ -9885,10 +9888,10 @@
     </row>
     <row r="15" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
@@ -9899,10 +9902,10 @@
     </row>
     <row r="16" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A16" s="14" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
@@ -9913,10 +9916,10 @@
     </row>
     <row r="17" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
@@ -9927,10 +9930,10 @@
     </row>
     <row r="18" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C18" s="14"/>
       <c r="D18" s="14"/>
@@ -9941,10 +9944,10 @@
     </row>
     <row r="19" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C19" s="14"/>
       <c r="D19" s="14"/>
@@ -10460,43 +10463,43 @@
         <v>101</v>
       </c>
       <c r="C1" s="29" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D1" s="29" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E1" s="29" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F1" s="29" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="G1" s="29" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H1" s="29" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="I1" s="29" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J1" s="29" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K1" s="29" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="L1" s="29" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="M1" s="29" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="N1" s="29" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="O1" s="29" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -10507,25 +10510,25 @@
         <v>112</v>
       </c>
       <c r="C2" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D2" t="s">
+        <v>264</v>
+      </c>
+      <c r="E2" t="s">
+        <v>265</v>
+      </c>
+      <c r="F2" t="s">
         <v>263</v>
       </c>
-      <c r="E2" t="s">
-        <v>264</v>
-      </c>
-      <c r="F2" t="s">
-        <v>262</v>
-      </c>
       <c r="G2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="H2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J2" t="s">
         <v>89</v>
@@ -10537,136 +10540,136 @@
         <v>92</v>
       </c>
       <c r="M2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="N2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="O2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C3" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="I3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="J3" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K3" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="L3" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="M3" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="N3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="O3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B4" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C4" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D4" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E4" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F4" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G4" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="I4" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K4" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="M4" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="N4" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="O4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B5" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C5" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D5" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E5" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F5" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G5" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="I5" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="K5" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="M5" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="N5" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="O5" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
@@ -10674,168 +10677,171 @@
         <v>108</v>
       </c>
       <c r="C6" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D6" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E6" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F6" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="K6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="M6" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="N6" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="O6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>369</v>
+        <v>370</v>
+      </c>
+      <c r="C7" t="s">
+        <v>117</v>
       </c>
       <c r="D7" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F7" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="M7" t="s">
         <v>88</v>
       </c>
       <c r="N7" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="O7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D8" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="M8" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="N8" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="O8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D9" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="M9" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="N9" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="O9" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D10" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="M10" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="N10" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="O10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="M11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="N11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="O11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="M12" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="N12" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="O12" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M13" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="N13" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="O13" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M14" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="N14" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="O14" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M15" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="N15" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="M16" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="N16" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>

</xml_diff>